<commit_message>
feat(rnaseq): add strandedness support and document multiple categories
- Add get_strandedness() function to extract per-sample strandedness
- Pass --rna-strandness RF/FR to HISAT2 based on Strandedness column
- Add Strandedness column to xlsx templates
- Document strandedness options (RF, FR, unstranded) in curator guide
- Document multiple categories support (comma-separated)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/rnaseq/RNA-seq_metadata_BLANK.xlsx
+++ b/docs/rnaseq/RNA-seq_metadata_BLANK.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -537,15 +537,20 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Strandedness</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Align_Pct</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>

</xml_diff>